<commit_message>
Allow max_count on fixed-add effects and include it in event data
Fixed-add types such as 初期評価 now accept max_count: 1 (or omitted);
any other value is an error since they always add once. The detail
table shows the value when given. Sample event entries carry
max_count, and docs, Excel help text and tests are updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FGf9edij8V2ChLtAAdoFDT
</commit_message>
<xml_diff>
--- a/excel/support_cards.xlsx
+++ b/excel/support_cards.xlsx
@@ -309,7 +309,7 @@
     <t>・今の計算式で表せない効果（パラメータ上昇量%アップ、条件付きの効果など）も空欄にしてください。</t>
   </si>
   <si>
-    <t>・固定加算の効果: 初期評価 … 行動回数に関係なく値を1回だけ加算します。最大回数は空欄にしてください。</t>
+    <t>・固定加算の効果: 初期評価 … 行動回数に関係なく値を1回だけ加算します。最大回数は 1 か空欄にしてください。</t>
   </si>
   <si>
     <t>・別の行動の回数で発動する効果: VoSP終了時（VoSPレッスンの回数） / DaSP終了時（DaSPレッスンの回数） / ViSP終了時（ViSPレッスンの回数）</t>
@@ -922,6 +922,9 @@
       <c r="H2" t="s">
         <v>45</v>
       </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
       <c r="J2">
         <v>20</v>
       </c>
@@ -1020,6 +1023,9 @@
       <c r="H3" t="s">
         <v>47</v>
       </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
       <c r="J3">
         <v>30</v>
       </c>
@@ -1219,6 +1225,9 @@
       <c r="H5" t="s">
         <v>47</v>
       </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
       <c r="J5">
         <v>10</v>
       </c>
@@ -1296,6 +1305,9 @@
       <c r="H6" t="s">
         <v>47</v>
       </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
       <c r="J6">
         <v>20</v>
       </c>
@@ -1394,6 +1406,9 @@
       <c r="H7" t="s">
         <v>50</v>
       </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
       <c r="J7">
         <v>30</v>
       </c>
@@ -1581,6 +1596,9 @@
       <c r="H9" t="s">
         <v>47</v>
       </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
       <c r="J9">
         <v>10</v>
       </c>
@@ -1655,6 +1673,9 @@
       <c r="H10" t="s">
         <v>50</v>
       </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
       <c r="J10">
         <v>20</v>
       </c>
@@ -1753,6 +1774,9 @@
       <c r="H11" t="s">
         <v>45</v>
       </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
       <c r="J11">
         <v>30</v>
       </c>
@@ -1939,6 +1963,9 @@
       </c>
       <c r="H13" t="s">
         <v>45</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
       </c>
       <c r="J13">
         <v>10</v>

</xml_diff>

<commit_message>
Rework action types: merged lessons, renamed types, new triggers
- Lessons: Vo/Da/Viレッスン now include SP lessons (SPレッスン inputs
  removed); Vo/Da/ViSP終了時 count from the matching lesson input
- 授業 -> 授業・営業終了時, 活動支給 -> 活動支給・差し入れ選択時
- Added 試験・オーディション終了時 and 好調/好印象/やる気/集中/元気/強気/
  温存/全力 効果カード獲得時 as inputs and effect types
- action_types.json entries can carry a description shown under the
  input name
- Sample data, Excel workbook (wider type column), README and tests
  updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FGf9edij8V2ChLtAAdoFDT
</commit_message>
<xml_diff>
--- a/excel/support_cards.xlsx
+++ b/excel/support_cards.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="111">
   <si>
     <t>ID</t>
   </si>
@@ -201,7 +201,7 @@
     <t>SR</t>
   </si>
   <si>
-    <t>授業</t>
+    <t>授業・営業終了時</t>
   </si>
   <si>
     <t>Voレッスン</t>
@@ -240,7 +240,7 @@
     <t>【サンプル】ダミーカードG</t>
   </si>
   <si>
-    <t>活動支給</t>
+    <t>活動支給・差し入れ選択時</t>
   </si>
   <si>
     <t>sample_008</t>
@@ -285,13 +285,31 @@
     <t>効果種類</t>
   </si>
   <si>
-    <t>VoSPレッスン</t>
-  </si>
-  <si>
-    <t>DaSPレッスン</t>
-  </si>
-  <si>
-    <t>ViSPレッスン</t>
+    <t>試験・オーディション終了時</t>
+  </si>
+  <si>
+    <t>好調効果カード獲得時</t>
+  </si>
+  <si>
+    <t>好印象効果カード獲得時</t>
+  </si>
+  <si>
+    <t>やる気効果カード獲得時</t>
+  </si>
+  <si>
+    <t>集中効果カード獲得時</t>
+  </si>
+  <si>
+    <t>元気効果カード獲得時</t>
+  </si>
+  <si>
+    <t>強気効果カード獲得時</t>
+  </si>
+  <si>
+    <t>温存効果カード獲得時</t>
+  </si>
+  <si>
+    <t>全力効果カード獲得時</t>
   </si>
   <si>
     <t>サポートカードデータ 入力シート</t>
@@ -312,10 +330,10 @@
     <t>・固定加算の効果: 初期評価 … 行動回数に関係なく値を1回だけ加算します。最大回数は 1 か空欄にしてください。</t>
   </si>
   <si>
-    <t>・別の行動の回数で発動する効果: VoSP終了時（VoSPレッスンの回数） / DaSP終了時（DaSPレッスンの回数） / ViSP終了時（ViSPレッスンの回数）</t>
-  </si>
-  <si>
-    <t>・上記以外の効果種類は、同じ名前の行動回数（Voレッスン / Daレッスン / Viレッスン / VoSPレッスン / DaSPレッスン / ViSPレッスン / 授業 / おでかけ / 相談 / 強化 / 削除 / 活動支給 / 休む）で発動します。</t>
+    <t>・別の行動の回数で発動する効果: VoSP終了時（Voレッスンの回数） / DaSP終了時（Daレッスンの回数） / ViSP終了時（Viレッスンの回数）</t>
+  </si>
+  <si>
+    <t>・上記以外の効果種類は、同じ名前の行動回数（Voレッスン / Daレッスン / Viレッスン / 授業・営業終了時 / おでかけ / 相談 / 活動支給・差し入れ選択時 / 強化 / 削除 / 休む / 試験・オーディション終了時 / 好調効果カード獲得時 / 好印象効果カード獲得時 / やる気効果カード獲得時 / 集中効果カード獲得時 / 元気効果カード獲得時 / 強気効果カード獲得時 / 温存効果カード獲得時 / 全力効果カード獲得時）で発動します。</t>
   </si>
   <si>
     <t>・イベント効果1〜2 は効果と同じ書き方（種類・対象・最大回数・値）で、計算方法も効果と同じです。なければ4列とも空欄にしてください。</t>
@@ -755,28 +773,28 @@
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
     <col min="8" max="8" width="7" customWidth="1"/>
     <col min="10" max="10" width="8" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="11" max="11" width="24" customWidth="1"/>
     <col min="12" max="12" width="7" customWidth="1"/>
     <col min="14" max="14" width="8" customWidth="1"/>
-    <col min="15" max="15" width="14" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
     <col min="16" max="16" width="7" customWidth="1"/>
     <col min="18" max="18" width="8" customWidth="1"/>
-    <col min="19" max="19" width="14" customWidth="1"/>
+    <col min="19" max="19" width="24" customWidth="1"/>
     <col min="20" max="20" width="7" customWidth="1"/>
     <col min="22" max="22" width="8" customWidth="1"/>
-    <col min="23" max="23" width="14" customWidth="1"/>
+    <col min="23" max="23" width="24" customWidth="1"/>
     <col min="24" max="24" width="7" customWidth="1"/>
     <col min="26" max="26" width="8" customWidth="1"/>
-    <col min="27" max="27" width="14" customWidth="1"/>
+    <col min="27" max="27" width="24" customWidth="1"/>
     <col min="28" max="28" width="7" customWidth="1"/>
     <col min="30" max="30" width="8" customWidth="1"/>
-    <col min="31" max="31" width="14" customWidth="1"/>
+    <col min="31" max="31" width="24" customWidth="1"/>
     <col min="32" max="32" width="7" customWidth="1"/>
     <col min="34" max="34" width="8" customWidth="1"/>
-    <col min="35" max="35" width="14" customWidth="1"/>
+    <col min="35" max="35" width="24" customWidth="1"/>
     <col min="36" max="36" width="7" customWidth="1"/>
     <col min="38" max="38" width="8" customWidth="1"/>
   </cols>
@@ -2019,7 +2037,7 @@
   </sheetData>
   <dataValidations count="34">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="AA2:AA1000">
-      <formula1>リスト!$C$2:$C$18</formula1>
+      <formula1>リスト!$C$2:$C$24</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="AB2:AB1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2031,7 +2049,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="AE2:AE1000">
-      <formula1>リスト!$C$2:$C$18</formula1>
+      <formula1>リスト!$C$2:$C$24</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="AF2:AF1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2043,7 +2061,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="AI2:AI1000">
-      <formula1>リスト!$C$2:$C$18</formula1>
+      <formula1>リスト!$C$2:$C$24</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="AJ2:AJ1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2061,7 +2079,7 @@
       <formula1>リスト!$D$2:$D$2</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="G2:G1000">
-      <formula1>リスト!$C$2:$C$18</formula1>
+      <formula1>リスト!$C$2:$C$24</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="H2:H1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2073,7 +2091,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="K2:K1000">
-      <formula1>リスト!$C$2:$C$18</formula1>
+      <formula1>リスト!$C$2:$C$24</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="L2:L1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2085,7 +2103,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="O2:O1000">
-      <formula1>リスト!$C$2:$C$18</formula1>
+      <formula1>リスト!$C$2:$C$24</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="P2:P1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2097,7 +2115,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="S2:S1000">
-      <formula1>リスト!$C$2:$C$18</formula1>
+      <formula1>リスト!$C$2:$C$24</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="T2:T1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2109,7 +2127,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="W2:W1000">
-      <formula1>リスト!$C$2:$C$18</formula1>
+      <formula1>リスト!$C$2:$C$24</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="X2:X1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2128,7 +2146,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2183,71 +2201,101 @@
     </row>
     <row r="5" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>90</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
-        <v>91</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>92</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>49</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>58</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>44</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
-        <v>51</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
-        <v>56</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C19" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
         <v>70</v>
       </c>
     </row>
@@ -2267,7 +2315,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2277,57 +2325,57 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 特別指導開始時 as an action input and effect type
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FGf9edij8V2ChLtAAdoFDT
</commit_message>
<xml_diff>
--- a/excel/support_cards.xlsx
+++ b/excel/support_cards.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="112">
   <si>
     <t>ID</t>
   </si>
@@ -285,6 +285,9 @@
     <t>効果種類</t>
   </si>
   <si>
+    <t>特別指導開始時</t>
+  </si>
+  <si>
     <t>試験・オーディション終了時</t>
   </si>
   <si>
@@ -333,7 +336,7 @@
     <t>・別の行動の回数で発動する効果: VoSP終了時（Voレッスンの回数） / DaSP終了時（Daレッスンの回数） / ViSP終了時（Viレッスンの回数）</t>
   </si>
   <si>
-    <t>・上記以外の効果種類は、同じ名前の行動回数（Voレッスン / Daレッスン / Viレッスン / 授業・営業終了時 / おでかけ / 相談 / 活動支給・差し入れ選択時 / 強化 / 削除 / 休む / 試験・オーディション終了時 / 好調効果カード獲得時 / 好印象効果カード獲得時 / やる気効果カード獲得時 / 集中効果カード獲得時 / 元気効果カード獲得時 / 強気効果カード獲得時 / 温存効果カード獲得時 / 全力効果カード獲得時）で発動します。</t>
+    <t>・上記以外の効果種類は、同じ名前の行動回数（Voレッスン / Daレッスン / Viレッスン / 授業・営業終了時 / おでかけ / 相談 / 活動支給・差し入れ選択時 / 強化 / 削除 / 休む / 特別指導開始時 / 試験・オーディション終了時 / 好調効果カード獲得時 / 好印象効果カード獲得時 / やる気効果カード獲得時 / 集中効果カード獲得時 / 元気効果カード獲得時 / 強気効果カード獲得時 / 温存効果カード獲得時 / 全力効果カード獲得時）で発動します。</t>
   </si>
   <si>
     <t>・イベント効果1〜2 は効果と同じ書き方（種類・対象・最大回数・値）で、計算方法も効果と同じです。なければ4列とも空欄にしてください。</t>
@@ -2037,7 +2040,7 @@
   </sheetData>
   <dataValidations count="34">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="AA2:AA1000">
-      <formula1>リスト!$C$2:$C$24</formula1>
+      <formula1>リスト!$C$2:$C$25</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="AB2:AB1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2049,7 +2052,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="AE2:AE1000">
-      <formula1>リスト!$C$2:$C$24</formula1>
+      <formula1>リスト!$C$2:$C$25</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="AF2:AF1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2061,7 +2064,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="AI2:AI1000">
-      <formula1>リスト!$C$2:$C$24</formula1>
+      <formula1>リスト!$C$2:$C$25</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="AJ2:AJ1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2079,7 +2082,7 @@
       <formula1>リスト!$D$2:$D$2</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="G2:G1000">
-      <formula1>リスト!$C$2:$C$24</formula1>
+      <formula1>リスト!$C$2:$C$25</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="H2:H1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2091,7 +2094,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="K2:K1000">
-      <formula1>リスト!$C$2:$C$24</formula1>
+      <formula1>リスト!$C$2:$C$25</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="L2:L1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2103,7 +2106,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="O2:O1000">
-      <formula1>リスト!$C$2:$C$24</formula1>
+      <formula1>リスト!$C$2:$C$25</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="P2:P1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2115,7 +2118,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="S2:S1000">
-      <formula1>リスト!$C$2:$C$24</formula1>
+      <formula1>リスト!$C$2:$C$25</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="T2:T1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2127,7 +2130,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「効果種類」の一覧から選んでください" sqref="W2:W1000">
-      <formula1>リスト!$C$2:$C$24</formula1>
+      <formula1>リスト!$C$2:$C$25</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="入力エラー" error="「対象」の一覧から選んでください" sqref="X2:X1000">
       <formula1>リスト!$B$2:$B$4</formula1>
@@ -2146,7 +2149,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2281,21 +2284,26 @@
     </row>
     <row r="21" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
-        <v>44</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C24" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
         <v>70</v>
       </c>
     </row>
@@ -2315,7 +2323,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2325,57 +2333,57 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>